<commit_message>
Updated IND_grids_kan model - 2026-05-13 19:24
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IND_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{96D31DE3-2441-422E-A788-AAE326D364F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{461A51A8-9165-4842-9C73-F90A29943C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6694,7 +6694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A03CCE75-B5F7-42F0-92E4-2C84833B2F4D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3363248E-E60A-4261-A4C2-D778AF91B34A}">
   <dimension ref="B9:H527"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -37267,7 +37267,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95DD79D7-1DFD-46C6-8C47-C63D236E8DDF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA0374E0-75F3-4B68-BB2A-193C70AA798C}">
   <dimension ref="B9:L527"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IND_grids_kan model - 2026-05-13 19:32
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IND_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{461A51A8-9165-4842-9C73-F90A29943C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AADA14FC-A910-49C6-A00C-0CAFC16C17A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6694,7 +6694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3363248E-E60A-4261-A4C2-D778AF91B34A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A77A081-38D5-4291-82BA-E5EE534E58EC}">
   <dimension ref="B9:H527"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -37267,7 +37267,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA0374E0-75F3-4B68-BB2A-193C70AA798C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9D14727-BF42-418C-B6AE-5F1AE2C52D40}">
   <dimension ref="B9:L527"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IND_grids_kan model - 2026-05-25 18:32
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IND_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AADA14FC-A910-49C6-A00C-0CAFC16C17A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7483AA38-80F6-4998-9937-661D7EA20212}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6694,7 +6694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A77A081-38D5-4291-82BA-E5EE534E58EC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{173AC544-CFED-46F3-ADCA-FCD5305E8FF6}">
   <dimension ref="B9:H527"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -37267,7 +37267,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9D14727-BF42-418C-B6AE-5F1AE2C52D40}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC981A98-C2EE-45FE-971A-AF8BFAD94957}">
   <dimension ref="B9:L527"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IND_grids_kan model - 2026-06-03 22:35
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IND_grids_kan/ReportDefs_vervestacks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7483AA38-80F6-4998-9937-661D7EA20212}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B56E0341-F974-4E82-BEE7-72529803C937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6694,7 +6694,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{173AC544-CFED-46F3-ADCA-FCD5305E8FF6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58C643C8-72C5-4CF5-A8BE-53E7B0D3D532}">
   <dimension ref="B9:H527"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -37267,7 +37267,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC981A98-C2EE-45FE-971A-AF8BFAD94957}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{583AF7D4-4150-4C51-9E14-DC6241BE583A}">
   <dimension ref="B9:L527"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>